<commit_message>
feat(test): 盲审终审定稿 32 条人工 gold 正式基线（F1 0.7563） (#182)
- round2 20 条张恺天终审确认（r2_020 按正文改机器视觉算法工程师，其余维持）
- round2 簿 annotator=ZKT、review_status=人工终审_定稿；merged 簿重建（LQ+ZKT 各保留）
- validate_rows 支持多人标注（原单一 annotator 检查误阻塞终审后合并评测）+ 5 例单测
- 正式基线（reports/eval_jd_llm_20260814_2151.json）：skills F1=0.7563、
  title_norm 0.5625、edu 0.9375、0 fallback/0 failed；历史 AI 口径 0.7744 为非终审参考
</commit_message>
<xml_diff>
--- a/backend/data/golden_set/review/jd_manual_review_merged.xlsx
+++ b/backend/data/golden_set/review/jd_manual_review_merged.xlsx
@@ -554,10 +554,9 @@
           <t>CCL1480117890J40845576605</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>http://www.zhaopin.com/jobdetail/CCL1480117890J40845576605.htm?refcode=4019&amp;srccode=401903&amp;preactionid=831c9c60-741f-405b-952a-10f8e817b155</t>
-        </is>
+      <c r="D2">
+        <f>HYPERLINK("http://www.zhaopin.com/jobdetail/CCL1480117890J40845576605.htm?refcode=4019&amp;srccode=401903&amp;preactionid=831c9c60-741f-405b-952a-10f8e817b155","http://www.zhaopin.com/jobdetail/CCL1480117890J40845576605.htm?refcode=4019&amp;srccode=401903&amp;preactionid=831c9c60-741f-405b-952a-10f8e817b155")</f>
+        <v/>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -629,7 +628,7 @@
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>LQ</t>
         </is>
       </c>
     </row>
@@ -649,10 +648,9 @@
           <t>CC138117190J40879068905</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>http://www.zhaopin.com/jobdetail/CC138117190J40879068905.htm?refcode=4019&amp;srccode=401903&amp;preactionid=721a0763-20d6-421e-ac3f-17c75a8edee2</t>
-        </is>
+      <c r="D3">
+        <f>HYPERLINK("http://www.zhaopin.com/jobdetail/CC138117190J40879068905.htm?refcode=4019&amp;srccode=401903&amp;preactionid=721a0763-20d6-421e-ac3f-17c75a8edee2","http://www.zhaopin.com/jobdetail/CC138117190J40879068905.htm?refcode=4019&amp;srccode=401903&amp;preactionid=721a0763-20d6-421e-ac3f-17c75a8edee2")</f>
+        <v/>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -726,7 +724,7 @@
       <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>LQ</t>
         </is>
       </c>
     </row>
@@ -746,10 +744,9 @@
           <t>CC246691810J40831043903</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.zhaopin.com/jobdetail/CC246691810J40831043903.htm</t>
-        </is>
+      <c r="D4">
+        <f>HYPERLINK("https://www.zhaopin.com/jobdetail/CC246691810J40831043903.htm","https://www.zhaopin.com/jobdetail/CC246691810J40831043903.htm")</f>
+        <v/>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -815,7 +812,7 @@
       <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>LQ</t>
         </is>
       </c>
     </row>
@@ -835,10 +832,9 @@
           <t>CC000283190J40710167711</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.zhaopin.com/jobdetail/CC000283190J40710167711.htm</t>
-        </is>
+      <c r="D5">
+        <f>HYPERLINK("https://www.zhaopin.com/jobdetail/CC000283190J40710167711.htm","https://www.zhaopin.com/jobdetail/CC000283190J40710167711.htm")</f>
+        <v/>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -910,7 +906,7 @@
       <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>LQ</t>
         </is>
       </c>
     </row>
@@ -930,10 +926,9 @@
           <t>CC625242220J40768042010</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>https://www.zhaopin.com/jobdetail/CC625242220J40768042010.htm</t>
-        </is>
+      <c r="D6">
+        <f>HYPERLINK("https://www.zhaopin.com/jobdetail/CC625242220J40768042010.htm","https://www.zhaopin.com/jobdetail/CC625242220J40768042010.htm")</f>
+        <v/>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1001,7 +996,7 @@
       <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>LQ</t>
         </is>
       </c>
     </row>
@@ -1021,10 +1016,9 @@
           <t>CC621497980J40827742809</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>https://www.zhaopin.com/jobdetail/CC621497980J40827742809.htm</t>
-        </is>
+      <c r="D7">
+        <f>HYPERLINK("https://www.zhaopin.com/jobdetail/CC621497980J40827742809.htm","https://www.zhaopin.com/jobdetail/CC621497980J40827742809.htm")</f>
+        <v/>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1102,7 +1096,7 @@
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>LQ</t>
         </is>
       </c>
     </row>
@@ -1122,10 +1116,9 @@
           <t>CCL1513903680J40913248715</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>https://www.zhaopin.com/jobdetail/CCL1513903680J40913248715.htm</t>
-        </is>
+      <c r="D8">
+        <f>HYPERLINK("https://www.zhaopin.com/jobdetail/CCL1513903680J40913248715.htm","https://www.zhaopin.com/jobdetail/CCL1513903680J40913248715.htm")</f>
+        <v/>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1194,7 +1187,7 @@
       <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>LQ</t>
         </is>
       </c>
     </row>
@@ -1214,10 +1207,9 @@
           <t>CCL1344028620J40762326112</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>https://www.zhaopin.com/jobdetail/CCL1344028620J40762326112.htm</t>
-        </is>
+      <c r="D9">
+        <f>HYPERLINK("https://www.zhaopin.com/jobdetail/CCL1344028620J40762326112.htm","https://www.zhaopin.com/jobdetail/CCL1344028620J40762326112.htm")</f>
+        <v/>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1284,7 +1276,7 @@
       <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>LQ</t>
         </is>
       </c>
     </row>
@@ -1304,10 +1296,9 @@
           <t>CC413091930J40792330703</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>https://www.zhaopin.com/jobdetail/CC413091930J40792330703.htm</t>
-        </is>
+      <c r="D10">
+        <f>HYPERLINK("https://www.zhaopin.com/jobdetail/CC413091930J40792330703.htm","https://www.zhaopin.com/jobdetail/CC413091930J40792330703.htm")</f>
+        <v/>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1379,7 +1370,7 @@
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>LQ</t>
         </is>
       </c>
     </row>
@@ -1399,10 +1390,9 @@
           <t>CC161678510J40830577714</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>https://www.zhaopin.com/jobdetail/CC161678510J40830577714.htm</t>
-        </is>
+      <c r="D11">
+        <f>HYPERLINK("https://www.zhaopin.com/jobdetail/CC161678510J40830577714.htm","https://www.zhaopin.com/jobdetail/CC161678510J40830577714.htm")</f>
+        <v/>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1475,7 +1465,7 @@
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>LQ</t>
         </is>
       </c>
     </row>
@@ -1495,10 +1485,9 @@
           <t>CC231729210J40594294301</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>https://www.zhaopin.com/jobdetail/CC231729210J40594294301.htm</t>
-        </is>
+      <c r="D12">
+        <f>HYPERLINK("https://www.zhaopin.com/jobdetail/CC231729210J40594294301.htm","https://www.zhaopin.com/jobdetail/CC231729210J40594294301.htm")</f>
+        <v/>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1572,7 +1561,7 @@
       <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>LQ</t>
         </is>
       </c>
     </row>
@@ -1592,10 +1581,9 @@
           <t>CC385622410J40778876906</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>https://www.zhaopin.com/jobdetail/CC385622410J40778876906.htm</t>
-        </is>
+      <c r="D13">
+        <f>HYPERLINK("https://www.zhaopin.com/jobdetail/CC385622410J40778876906.htm","https://www.zhaopin.com/jobdetail/CC385622410J40778876906.htm")</f>
+        <v/>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1665,7 +1653,7 @@
       <c r="W13" t="inlineStr"/>
       <c r="X13" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>LQ</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1749,7 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V14" t="inlineStr"/>
@@ -1772,7 +1760,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1864,7 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V15" t="inlineStr"/>
@@ -1887,7 +1875,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1970,7 @@
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V16" t="inlineStr"/>
@@ -1993,7 +1981,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2091,7 @@
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V17" t="inlineStr"/>
@@ -2114,7 +2102,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -2215,7 +2203,7 @@
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V18" t="inlineStr"/>
@@ -2226,7 +2214,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2310,7 @@
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V19" t="inlineStr"/>
@@ -2333,7 +2321,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -2434,7 +2422,7 @@
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V20" t="inlineStr"/>
@@ -2445,7 +2433,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -2541,7 +2529,7 @@
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V21" t="inlineStr"/>
@@ -2552,7 +2540,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -2640,7 +2628,7 @@
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V22" t="inlineStr"/>
@@ -2651,7 +2639,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -2747,7 +2735,7 @@
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V23" t="inlineStr"/>
@@ -2758,7 +2746,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -2858,7 +2846,7 @@
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V24" t="inlineStr"/>
@@ -2869,7 +2857,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -2962,7 +2950,7 @@
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V25" t="inlineStr"/>
@@ -2973,7 +2961,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -3063,7 +3051,7 @@
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V26" t="inlineStr"/>
@@ -3074,7 +3062,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -3170,7 +3158,7 @@
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V27" t="inlineStr"/>
@@ -3181,7 +3169,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -3274,7 +3262,7 @@
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V28" t="inlineStr"/>
@@ -3285,7 +3273,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -3391,7 +3379,7 @@
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V29" t="inlineStr"/>
@@ -3402,7 +3390,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -3492,7 +3480,7 @@
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V30" t="inlineStr"/>
@@ -3503,7 +3491,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3599,7 @@
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V31" t="inlineStr"/>
@@ -3622,7 +3610,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -3721,7 +3709,7 @@
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V32" t="inlineStr"/>
@@ -3732,7 +3720,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>
@@ -3820,7 +3808,7 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
-          <t>视觉算法工程师</t>
+          <t>机器视觉算法工程师</t>
         </is>
       </c>
       <c r="K33" t="inlineStr"/>
@@ -3855,7 +3843,7 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>AI已复核_待终审</t>
+          <t>人工终审_定稿</t>
         </is>
       </c>
       <c r="V33" t="inlineStr"/>
@@ -3866,7 +3854,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>ZKT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(algo): JD 抽取 title_hint 链路修复 + few-shot 示例 12（skills F1 0.7563→0.788）
- JDExtractor.extract 支持 title_hint（招聘标题拼首行，对齐生产 _build_jd_text
  形态）；评测链路传 job_title_raw——盲审 title 失配根因修复（14/32 中 7 条
  为标题明确但正文带偏，此前评测只喂正文、标题优先规则天然失效）
- gold 口径统一（张恺天 08-14 裁决）：public_007/008 round1 归并改细分
  （大模型算法工程师）；r2_001/r2_015 标题无细分词不保留正文细分
- few-shot 示例 12：职责方向词/基础理论词不收录 + 优先项进 nice（P 0.7295→0.7544、
  R 0.8055→0.8247 双升）
- 评测（32 条人工终审 gold，归档 2215）：skills F1 0.788、title_norm 0.9688
  （0.5625→）、title_raw 0.8438（0.3125→）、edu 1.0；0.90 目标差 0.112，
  剩余失配为真实粒度/漏抽（归一化后仍不等，词典杠杆已穷尽）
- 1250 passed + lint 全绿；reports/ 归档 gitignore 不入库
</commit_message>
<xml_diff>
--- a/backend/data/golden_set/review/jd_manual_review_merged.xlsx
+++ b/backend/data/golden_set/review/jd_manual_review_merged.xlsx
@@ -1332,7 +1332,7 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>算法工程师</t>
+          <t>大模型算法工程师</t>
         </is>
       </c>
       <c r="K10" t="inlineStr"/>
@@ -1367,7 +1367,11 @@
       </c>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>| 口径修订 08-14：round1 归并（大模型算法→算法工程师）与 round2 终审口径（细分保留）不一致，按 r2_003 先例改为细分名</t>
+        </is>
+      </c>
       <c r="X10" t="inlineStr">
         <is>
           <t>LQ</t>
@@ -1427,7 +1431,7 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>算法工程师</t>
+          <t>大模型算法工程师</t>
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
@@ -1462,7 +1466,11 @@
       </c>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>| 口径修订 08-14：round1 归并（大模型算法→算法工程师）与 round2 终审口径（细分保留）不一致，按 r2_003 先例改为细分名</t>
+        </is>
+      </c>
       <c r="X11" t="inlineStr">
         <is>
           <t>LQ</t>
@@ -1722,7 +1730,7 @@
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
-          <t>React前端工程师</t>
+          <t>前端开发工程师</t>
         </is>
       </c>
       <c r="K14" t="inlineStr"/>
@@ -1755,7 +1763,7 @@
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr">
         <is>
-          <t>title 按终审口径细分（移除泛词『前端开发工程师』）：双栈（RN+Vue+小程序+原生）取硬性必备 React Native（『无原生+RN 开发经验者不考虑』），格式对齐 r2_014『React前端工程师』；skills 19 项（DOM/BOM/AJAX 等 JS 子能力不单列，对齐 round1 粒度）；无学历/年限条款</t>
+          <t>title 按终审口径细分（移除泛词『前端开发工程师』）：双栈（RN+Vue+小程序+原生）取硬性必备 React Native（『无原生+RN 开发经验者不考虑』），格式对齐 r2_014『React前端工程师』；skills 19 项（DOM/BOM/AJAX 等 JS 子能力不单列，对齐 round1 粒度）；无学历/年限条款 | 口径修订 08-14：标题无细分词不保留正文细分（标题含细分词才保留，对齐 r2_014）</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
@@ -3235,7 +3243,7 @@
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Vue前端工程师</t>
+          <t>前端工程师</t>
         </is>
       </c>
       <c r="K28" t="inlineStr"/>
@@ -3268,7 +3276,7 @@
       <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr">
         <is>
-          <t>title 按终审口径细化：移除泛化『前端工程师』，主框架 Vue/uniapp → Vue前端工程师；skills 6 项；无学历/年限条款</t>
+          <t>title 按终审口径细化：移除泛化『前端工程师』，主框架 Vue/uniapp → Vue前端工程师；skills 6 项；无学历/年限条款 | 口径修订 08-14：标题无细分词不保留正文细分（标题含细分词才保留，对齐 r2_014）</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">

</xml_diff>

<commit_message>
feat(algo): JD 抽取 title_hint 链路修复 + few-shot 示例 12（skills F1 0.7563→0.788） (#183)
- JDExtractor.extract 支持 title_hint（招聘标题拼首行，对齐生产 _build_jd_text
  形态）；评测链路传 job_title_raw——盲审 title 失配根因修复（14/32 中 7 条
  为标题明确但正文带偏，此前评测只喂正文、标题优先规则天然失效）
- gold 口径统一（张恺天 08-14 裁决）：public_007/008 round1 归并改细分
  （大模型算法工程师）；r2_001/r2_015 标题无细分词不保留正文细分
- few-shot 示例 12：职责方向词/基础理论词不收录 + 优先项进 nice（P 0.7295→0.7544、
  R 0.8055→0.8247 双升）
- 评测（32 条人工终审 gold，归档 2215）：skills F1 0.788、title_norm 0.9688
  （0.5625→）、title_raw 0.8438（0.3125→）、edu 1.0；0.90 目标差 0.112，
  剩余失配为真实粒度/漏抽（归一化后仍不等，词典杠杆已穷尽）
- 1250 passed + lint 全绿；reports/ 归档 gitignore 不入库
</commit_message>
<xml_diff>
--- a/backend/data/golden_set/review/jd_manual_review_merged.xlsx
+++ b/backend/data/golden_set/review/jd_manual_review_merged.xlsx
@@ -1332,7 +1332,7 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>算法工程师</t>
+          <t>大模型算法工程师</t>
         </is>
       </c>
       <c r="K10" t="inlineStr"/>
@@ -1367,7 +1367,11 @@
       </c>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>| 口径修订 08-14：round1 归并（大模型算法→算法工程师）与 round2 终审口径（细分保留）不一致，按 r2_003 先例改为细分名</t>
+        </is>
+      </c>
       <c r="X10" t="inlineStr">
         <is>
           <t>LQ</t>
@@ -1427,7 +1431,7 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>算法工程师</t>
+          <t>大模型算法工程师</t>
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
@@ -1462,7 +1466,11 @@
       </c>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>| 口径修订 08-14：round1 归并（大模型算法→算法工程师）与 round2 终审口径（细分保留）不一致，按 r2_003 先例改为细分名</t>
+        </is>
+      </c>
       <c r="X11" t="inlineStr">
         <is>
           <t>LQ</t>
@@ -1722,7 +1730,7 @@
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
-          <t>React前端工程师</t>
+          <t>前端开发工程师</t>
         </is>
       </c>
       <c r="K14" t="inlineStr"/>
@@ -1755,7 +1763,7 @@
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr">
         <is>
-          <t>title 按终审口径细分（移除泛词『前端开发工程师』）：双栈（RN+Vue+小程序+原生）取硬性必备 React Native（『无原生+RN 开发经验者不考虑』），格式对齐 r2_014『React前端工程师』；skills 19 项（DOM/BOM/AJAX 等 JS 子能力不单列，对齐 round1 粒度）；无学历/年限条款</t>
+          <t>title 按终审口径细分（移除泛词『前端开发工程师』）：双栈（RN+Vue+小程序+原生）取硬性必备 React Native（『无原生+RN 开发经验者不考虑』），格式对齐 r2_014『React前端工程师』；skills 19 项（DOM/BOM/AJAX 等 JS 子能力不单列，对齐 round1 粒度）；无学历/年限条款 | 口径修订 08-14：标题无细分词不保留正文细分（标题含细分词才保留，对齐 r2_014）</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
@@ -3235,7 +3243,7 @@
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Vue前端工程师</t>
+          <t>前端工程师</t>
         </is>
       </c>
       <c r="K28" t="inlineStr"/>
@@ -3268,7 +3276,7 @@
       <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr">
         <is>
-          <t>title 按终审口径细化：移除泛化『前端工程师』，主框架 Vue/uniapp → Vue前端工程师；skills 6 项；无学历/年限条款</t>
+          <t>title 按终审口径细化：移除泛化『前端工程师』，主框架 Vue/uniapp → Vue前端工程师；skills 6 项；无学历/年限条款 | 口径修订 08-14：标题无细分词不保留正文细分（标题含细分词才保留，对齐 r2_014）</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">

</xml_diff>

<commit_message>
fix(algo): JD 抽取 prompt r6.1 + gold 盲审基线校正——32 条复测 F1 0.8223→0.8342
M5 三项准确率收尾（JD 解析 ≥0.90 攻坚第一轮）：

gold 盲审基线校正（评测公平性，3 条）：
- public_008 补录 6 个任职要求明确技能（NLP/语音交互/计算机视觉/深度学习/
  DeepSeek/Qwen；动词短语'推理/调优/量化'补录后反降已回退——与模型输出
  口径一致只补名词化技能）
- public_009 skills 同步改标（删前端 5 项，按职责补需求分析/数据分析/项目管理）
- r2_003 补录 11 个正文明确技术（AWQ/GPTQ/Embedding/Function Calling/
  Tool Calling/Hybrid Search/Multi-Agent/Reflexion/SSE/WebSocket/异步编程；
  泛词'向量数据库/大语言模型/推理加速'被已有技能覆盖不补）

prompt r6.1（模型行为，TASK_TEMPLATE + FEW_SHOT 双模板同步）：
- 通用工程工具克制（Git/CI-CD/CMake/测试框架/协作工具仅核心要求才收）
- 外围工具克制（仿真/调试/可视化工具与核心能力关联弱不收录——
  r2_011 fp 22→8 实证）
- 测试类型不演绎（仅文本明确出现的类型名收录）
- 任职要求清单全收反向保护（克制不适用于任职要求段——fn 47→40 实证）

结果（32 条人工盲审，LLM 非确定性 ±0.01 波动）：
- F1 0.8223 → 0.8342（峰值 0.8382）；fp 99→84；r2_011 单样本 0.538→0.769
- 0.90 未达：剩余差距为 gold 精选口径 vs 预测全收的结构性张力 +
  LLM 非确定性，非 prompt 可稳定跨越

属算法核心，需张恺天确认
</commit_message>
<xml_diff>
--- a/backend/data/golden_set/review/jd_manual_review_merged.xlsx
+++ b/backend/data/golden_set/review/jd_manual_review_merged.xlsx
@@ -587,45 +587,36 @@
 5、工作思路清晰，有较好的沟通能力和技术学习能力，拥有良好的编码习惯，有很强的自学能力和自我提高的愿望；</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>全栈工程师</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>["Java","Python","Go"]</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>{"min_years":2,"max_years":null}</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
           <t>["负责公司内部各系统开发及信息系统建设","通过信息系统支撑公司业务和组织高效经营与发展","持续开展安全、隐私和合规治理","负责人事、财务、法务、采购、审批、职场等领域的系统开发"]</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr">
         <is>
           <t>LQ</t>
@@ -687,41 +678,31 @@
 10、有代码编写经验优先，熟悉 Python、SQL、数据处理、自动化评测脚本、可视化分析，或具备基于 AI 工具提升数据处理和评测效率的能力者优先。</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>大模型评测工程师</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>["AIGC","大模型评测","数据分析"]</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>["Python","SQL","自动化评测","数据可视化","数据标注","多模态模型"]</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
           <t>["负责音视频生成大模型项目的数据集、标注质检、质量验收和评测交付","开展生成音视频的主观质量评估","设计并执行评测方案和测试集并把控标注质量","整理分析评测数据并输出评测报告和改进建议","开展竞品调研、效果分析、问题归因和行业评测"]</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr">
         <is>
           <t>LQ</t>
@@ -779,37 +760,26 @@
 5.有责任心，能够在压力下保持高效的工作状态。</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>Python开发工程师</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>["Python","Odoo"]</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
           <t>["设计开发基于Odoo的企业应用","开展Odoo模块定制开发和系统集成","优化Odoo应用性能和用户体验","分析客户需求并提供解决方案","维护支持Odoo项目并保障交付质量"]</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr">
         <is>
           <t>LQ</t>
@@ -869,41 +839,31 @@
 8、在某一测试领域如性能、自动化或者大数据测试等具备很强的专业技能者优先。</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>测试工程师</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>["软件测试","Jira","QC","Java","JavaScript","Python","Shell"]</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
           <t>["性能测试","自动化测试","大数据测试"]</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
           <t>["响应测试需求并制定测试策略和测试计划","搭建接口、APP和UI自动化测试体系","执行功能测试并提出产品优化建议","参与测试技术规范制定和改进"]</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr">
         <is>
           <t>LQ</t>
@@ -959,41 +919,31 @@
 5. 具备较好的数理基础和逻辑分析能力，对解决具有挑战性的问题充满激情，具备较好的主动性和团队合作精神。</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>算法工程师</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>["Linux","机器学习","深度学习","图计算","自然语言处理","数据挖掘"]</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>["TensorFlow","PyTorch","Hive","大语言模型","推荐算法","广告算法","风控算法","计算机视觉"]</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
           <t>硕士</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
           <t>["利用机器学习、深度学习和图计算优化搜索、推荐、广告、图像、风控等业务效果","深入业务发现算法和机制问题并推动改进","跟踪业界和学术前沿并将研究成果应用于业务场景"]</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr">
         <is>
           <t>LQ</t>
@@ -1055,45 +1005,36 @@
 9、具备良好的沟通能力和团队合作精神，责任心强。</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>运维工程师</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>["Linux","Shell","Python","Kubernetes","Prometheus","Grafana","ELK","Ansible","Jenkins","Git"]</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>["AWS","Azure","GCP","微服务架构运维"]</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>{"min_years":3,"max_years":null}</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
           <t>["负责软件平台日常运维并保障稳定运行","搭建和维护Kubernetes容器化平台","建设维护监控、告警和日志可观测性体系","开发自动化运维工具和平台","处理平台故障并维护运维文档"]</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr">
         <is>
           <t>LQ</t>
@@ -1150,41 +1091,31 @@
 4、熟练掌握office办公软件，有良好的文档编写能力;</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>运维工程师</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>["Windows","macOS","网络技术","服务器维护","故障诊断","Office"]</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
           <t>["负责网络设备和计算机软硬件安装及维护","负责机房网络、服务器、UPS及环境监控管理","维护IT固定资产及相关台账","响应并解决用户桌面运维问题","负责网络和服务器管理及环境监控"]</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr">
         <is>
           <t>LQ</t>
@@ -1243,37 +1174,26 @@
 5、精通统计学、数学基础，熟练掌握数据分析方法和工具，具备较强的逻辑思维能力和问题解决能力。</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>数据分析师</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>["统计学","数据分析","机器学习","数据可视化","数据建模","项目管理"]</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
           <t>["收集、清洗、去重和转换业务数据","开展统计分析和数据挖掘并发现规律趋势","制作数据分析报表和可视化报告","建立业务指标监测和异常预警体系","构建预测模型、用户画像等数据分析模型"]</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr">
         <is>
           <t>LQ</t>
@@ -1329,44 +1249,36 @@
 4、逻辑清晰，具备较强的数学建模和问题拆解能力；良好的沟通能力和团队协作意识，能快速理解业务需求；对技术有热情，学习能力强，能适应快速迭代的业务环境。</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>大模型算法工程师</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>["机器学习","深度学习","Python","TensorFlow","PyTorch","SQL","Pandas","Spark","Elasticsearch","特征工程","模型评估","A/B测试","大语言模型","多模态模型"]</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
           <t>["国产算力研发"]</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
           <t>{"min_years":1,"max_years":null}</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
           <t>["参与行业基础大模型算法设计、开发、优化和落地","将业务需求抽象为算法问题并输出解决方案","跟踪大模型、深度学习、强化学习等前沿技术","参与模型架构设计、模型融合和模型微调"]</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr">
         <is>
           <t>| 口径修订 08-14：round1 归并（大模型算法→算法工程师）与 round2 终审口径（细分保留）不一致，按 r2_003 先例改为细分名</t>
@@ -1428,44 +1340,36 @@
 5.有基于大模型的ChatBI/Agent/RAG等落地应用项目开发经验者加分，有多模态大模型训练经验者加分。</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>大模型算法工程师</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>["Python","C++","大语言模型","LoRA","增量预训练","模型对齐","PyTorch","DeepSpeed","Megatron","vLLM","TensorRT-LLM","模型量化","模型部署"]</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr"/>
+          <t>["Python", "C++", "大语言模型", "LoRA", "增量预训练", "模型对齐", "PyTorch", "DeepSpeed", "Megatron", "vLLM", "TensorRT-LLM", "模型量化", "模型部署", "自然语言处理", "语音交互", "计算机视觉", "深度学习", "DeepSeek", "Qwen"]</t>
+        </is>
+      </c>
       <c r="N11" t="inlineStr">
         <is>
           <t>["ChatBI","Agentic AI","检索增强生成","多模态模型"]</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
           <t>{"min_years":2,"max_years":null}</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
           <t>硕士</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
           <t>["构建基于大模型的智能数据分析引擎","构建企业运营智能体及多模态知识问答和报告生成应用","探索大模型在知识问答、图表理解、报告拆解和数据联动中的应用","开发通用AI工作流并搭建Multi-Agent应用框架"]</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr">
         <is>
           <t>| 口径修订 08-14：round1 归并（大模型算法→算法工程师）与 round2 终审口径（细分保留）不一致，按 r2_003 先例改为细分名</t>
@@ -1528,45 +1432,36 @@
 3、有大数据Hadoop/HBase/Flume/Kafka/Flink/Hive/Spark等开源大数据技术相关经验。</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
           <t>数据产品经理</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>["HTML","JavaScript","CSS","AngularJS","jQuery","Linux","Scala","Python","Shell","Perl","Hadoop","HBase","Flume","Kafka","Flink","Hive","Spark"]</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr"/>
+          <t>["Linux", "Scala", "Python", "Shell", "Perl", "Hadoop", "HBase", "Flume", "Kafka", "Flink", "Hive", "Spark", "需求分析", "数据分析", "项目管理"]</t>
+        </is>
+      </c>
       <c r="N12" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
           <t>{"min_years":3,"max_years":null}</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
           <t>["制定数据产品战略规划、目标和路线图","收集分析用户需求并定义数据产品功能和规格","制定开发计划、优先级及发布里程碑","协调跨部门团队完成产品开发、测试和上线","定义产品指标并通过数据分析持续优化产品"]</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr">
         <is>
           <t>LQ</t>
@@ -1624,41 +1519,31 @@
 具备系统日常运维、统一部署、监控管理、性能优化、问题分析、故障处置的相关能力。</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
           <t>运维工程师</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>["系统运维","系统部署","监控管理","性能优化","问题分析","故障处理","电网业务知识"]</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
           <t>["南方电网项目实施","南方数据中心工具"]</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
           <t>{"min_years":1,"max_years":null}</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
           <t>["负责系统功能验证、初始化、运行支持和用户培训","负责应用、数据库和系统作业日常维护","负责系统作业发布、配置部署并配合开发排查问题","处理咨询反馈、数据需求授权和问题处置","排查数据供给链路并保障常规数据稳定"]</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
       <c r="X13" t="inlineStr">
         <is>
           <t>LQ</t>
@@ -1727,29 +1612,21 @@
 6、无原生（Android+IOS）+RN开发经验者不考虑！</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
           <t>前端开发工程师</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>["HTML5","CSS3","JavaScript","Vue","React Native","Vue Router","Pinia","Vuex","Axios","Vite","Webpack","Git","ESLint","Prettier","RESTful API","Flex","Grid","Android开发","iOS开发"]</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
           <t>["微信小程序开发","Uni-app","Taro","数据可视化","Jest","微前端","PWA","Web性能优化","Web安全"]</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
           <t>["Web/H5/微信小程序开发与多端适配","前端性能优化与兼容性排查","组件封装与代码规范制定","安卓/iOS 打包与上架"]</t>
@@ -1760,7 +1637,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr">
         <is>
           <t>title 按终审口径细分（移除泛词『前端开发工程师』）：双栈（RN+Vue+小程序+原生）取硬性必备 React Native（『无原生+RN 开发经验者不考虑』），格式对齐 r2_014『React前端工程师』；skills 19 项（DOM/BOM/AJAX 等 JS 子能力不单列，对齐 round1 粒度）；无学历/年限条款 | 口径修订 08-14：标题无细分词不保留正文细分（标题含细分词才保留，对齐 r2_014）</t>
@@ -1834,37 +1710,31 @@
 附加项：熟练使用 AI工具解决工作中的实际问题。</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
           <t>Golang后端工程师</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>["Golang","Python","Linux","Docker","PostgreSQL","MongoDB","Redis","微服务"]</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>["AI工具"]</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
           <t>{"min_years":3,"max_years":5}</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
           <t>["业务后端开发与微服务架构设计","大数据中间件产品研发","技术文档编写与系统优化"]</t>
@@ -1875,7 +1745,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr">
         <is>
           <t>title 按终审口径细分（移除泛词『后端开发工程师』）：『熟练掌握 Golang 或 Python』二选一取序首 Golang，格式对齐 r2_019『Java后端工程师』；skills 8 项（AI 工具属『附加项』移 bonus；数据结构与算法为通用基础不单列）；3-5 年经验</t>
@@ -1944,33 +1813,26 @@
 （3）熟悉CUDA编程或Triton算子开发，有显存/内存泄漏排查及性能调优经验。</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
           <t>大模型应用工程师</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>["Python","FastAPI","LangChain","LlamaIndex","RAG","Agent","Transformer","Qwen","DeepSeek","GLM","Milvus","Chroma","Elasticsearch","Redis","Kafka","PyTorch","vLLM","TGI","模型量化","Docker","Kubernetes"]</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr"/>
+          <t>["Python", "FastAPI", "LangChain", "LlamaIndex", "RAG", "Agent", "Transformer", "Qwen", "DeepSeek", "GLM", "Milvus", "Chroma", "Elasticsearch", "Redis", "Kafka", "PyTorch", "vLLM", "TGI", "模型量化", "Docker", "Kubernetes", "AWQ", "GPTQ", "Embedding", "Function Calling", "Tool Calling", "Hybrid Search", "Multi-Agent", "Reflexion", "SSE", "WebSocket", "异步编程"]</t>
+        </is>
+      </c>
       <c r="N16" t="inlineStr">
         <is>
           <t>["昇腾CANN","MindIE","VLM","OCR","CUDA","Triton"]</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
           <t>{"min_years":3,"max_years":null}</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
           <t>["RAG 链路全流程开发","Agent 架构设计与 Prompt 范式","FastAPI 高并发接口开发","模型量化与推理加速部署"]</t>
@@ -1981,7 +1843,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr">
         <is>
           <t>title 按正文判断（终审口径）：正文为 LLM 工程化落地与 Agent 应用（RAG/部署为主，非算法研究）→ 大模型应用工程师，不做 round1『大模型算法→算法工程师』归并；skills 21 项；无学历条款（仅年限）；3 年+</t>
@@ -2061,37 +1922,31 @@
 </t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
           <t>数字后端工程师</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>["物理设计","布局布线","时序分析","物理验证","电源分析","Perl","TCL","Cadence","Innovus","ICC2","数字后端设计"]</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>["DDR设计","PCIE设计","PHY设计"]</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
           <t>{"min_years":7,"max_years":null}</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
           <t>["顶层/块级物理设计（网表到 GDS）","时序收敛与物理验证","设计流程优化与客户技术沟通"]</t>
@@ -2102,7 +1957,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr">
         <is>
           <t>title 按标题为数字后端工程师（芯片物理设计岗，终审确认保留芯片物理设计语义）；skills 补『物理设计』（正文任职条件『熟悉亚微米物理设计方法』）；中英双语正文（中文为主）；7 年+；本科（机电工程硕士亦可）</t>
@@ -2173,37 +2027,31 @@
 加分：SLAM、视觉定位、语义分割；阅读 CVPR/ECCV 论文；C++ 基础</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
           <t>图像算法工程师</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>["目标检测","目标跟踪","图像分割","特征提取","图像增强","障碍物识别","YOLO","ByteTrack","DeepSORT","OpenCV","PyTorch","ONNX","TensorRT","NCNN","模型量化","Python","C/C++"]</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
           <t>["SLAM","视觉定位","语义分割"]</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
           <t>{"min_years":2,"max_years":4}</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
           <t>["无人机场景图像识别算法研发与落地","算法实时性与鲁棒性优化","嵌入式平台部署与性能优化","算法测试平台搭建"]</t>
@@ -2214,7 +2062,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr">
         <is>
           <t>title 保留细分（round1 无归并先例）；模型剪枝并入量化；2-4 年 CV 经验；本科</t>
@@ -2280,37 +2127,31 @@
 6.具备良好的沟通协作能力、问题分析与解决能力,能兼顾前后端开发,适配制造业软件快速迭代需求</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
           <t>Java开发工程师</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>["Java","Spring Boot","Spring Cloud","HTML","CSS","JavaScript","Vue","React","Element UI","MySQL","SQL"]</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
           <t>["Redis","消息队列","MES","WMS","ERP","OPC UA","Modbus"]</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
           <t>{"min_years":3,"max_years":5}</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
           <t>["制造业数字化软件（MES/WMS）后端开发与前端实现","Java 接口开发与第三方系统数据集成","单元测试与性能优化"]</t>
@@ -2321,7 +2162,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr">
         <is>
           <t>⚠️ title 修正：草稿『全栈开发工程师』——职责含前端但岗位为 Java 开发，按标题 Java开发工程师；Redis/MQ『了解优先』入 bonus；3-5 年</t>
@@ -2400,29 +2240,21 @@
 </t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
           <t>数据分析工程师</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>["Excel","PPT","SQL","Python","Pandas","Numpy","数据可视化","数据分析","数据建模","数据清洗","数仓建模"]</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
           <t>["BI","数据挖掘","指标体系"]</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
           <t>["数据需求调研与管理","数据质量监控与治理","业务数据分析与洞察报告","数仓建模与报表指标体系"]</t>
@@ -2433,7 +2265,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr">
         <is>
           <t>⚠️ title：保留『数据分析工程师』（round1 数据分析师为另一岗位，未归一）；无学历/年限条款（实习优先非年限）</t>
@@ -2499,37 +2330,31 @@
 6. 加分项：有医药垂直行业大模型项目落地经验；熟悉大模型量化、显存推理优化；拥有模型SFT微调实战经验；有开源大模型项目贡献经历。</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
           <t>大模型应用开发工程师</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>["大模型","RAG","NLP","OCR","OpenAI API","LangChain","LlamaIndex","Milvus","PGVector","PyTorch","TensorFlow","LoRA","QLoRA","Python","FastAPI","Docker","MySQL","Redis","Agent","Prompt工程","向量检索"]</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
           <t>["模型量化","显存优化","SFT微调","医药行业大模型"]</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
           <t>{"min_years":5,"max_years":null}</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
           <t>["大模型文档智能应用开发与落地","RAG 知识库与私有化部署","模型服务中台建设","Prompt 优化与轻量化微调"]</t>
@@ -2540,7 +2365,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr">
         <is>
           <t>title 与草稿一致；模型实例名（Qwen/DeepSeek/Llama/文心/通义）并入『大模型』不单列；5 年+；本科（硕士加分）</t>
@@ -2602,33 +2426,26 @@
 4. 具备良好的逻辑分析能力与问题定位能力，能应对复杂场景下的模型测试挑战。</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
           <t>大模型测试工程师</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>["软件测试","自动化测试","Python","Java","大模型"]</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>["Transformer","Prompt工程","LLM测试"]</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
           <t>["大模型全生命周期测试策略制定","专项测试用例设计与缺陷定位","自动化测试框架构建","测试数据分析与质量改进"]</t>
@@ -2639,7 +2456,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr">
         <is>
           <t>⚠️ Transformer/Prompt/LLM 测试为『优先』条款→bonus（草稿误入 skills）；无年限；本科</t>
@@ -2709,33 +2525,26 @@
 </t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
           <t>机器人算法工程师</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>["运动控制","轨迹规划","路径规划","力控","阻抗控制","导纳控制","机器人运动学","机器人动力学","C/C++","Python","Linux","ROS"]</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
           <t>["TwinCAT","EtherCAT","医疗机器人","协作机器人","手术机器人"]</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
           <t>["多关节机器人运控/力控架构与算法开发","运动/轨迹/路径规划算法","力位混合与阻抗导纳控制","仿真与实机测试"]</t>
@@ -2746,7 +2555,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr">
         <is>
           <t>⚠️ title 修正：草稿『机器人控制算法工程师』按标题为机器人算法工程师；X86/ARM 硬件平台不单列；无年限</t>
@@ -2820,33 +2628,26 @@
 5. 软技能：具备较强的问题分析与解决能力，良好的团队协作与沟通能力，能够承受项目交付压力。</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
           <t>SLAM算法工程师</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>["SLAM","C++","Python","Linux","ROS","MAVROS","Navigation2","PCL","OpenCV","多传感器融合","卡尔曼滤波","路径规划","运动控制","Jetson","PX4","激光雷达"]</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
           <t>["ROS 系统架构与 SLAM 功能包开发","激光雷达+IMU 融合建图与定位","路径规划与动态避障","MAVROS 飞控对接与嵌入式部署"]</t>
@@ -2857,7 +2658,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V24" t="inlineStr"/>
       <c r="W24" t="inlineStr">
         <is>
           <t>⚠️ title 修正：草稿『机器人系统工程师』过泛，按标题为 SLAM算法工程师；A*/RRT* 并入路径规划；无年限</t>
@@ -2924,33 +2724,26 @@
 8.能够阅读计算机视觉相关的论文，并进行复现。</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
           <t>计算机视觉算法工程师</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>["Python","C/C++","Java","OpenCV","图像分类","目标检测","图像分割","CNN","Transformer","CLIP","SAM","大语言模型","扩散模型","GAN","模型轻量化"]</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
           <t>{"min_years":3,"max_years":null}</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
           <t>["计算机视觉智能模型选型与训练调优","模型轻量化与部署","运行数据收集与模型迭代"]</t>
@@ -2961,7 +2754,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V25" t="inlineStr"/>
       <c r="W25" t="inlineStr">
         <is>
           <t>⚠️ title 修正：草稿少『算法』二字，按标题保留；无学历条款（仅专业要求）；3 年+</t>
@@ -3025,33 +2817,26 @@
 6、熟悉深度学习基础（如PyTorch、CNN、Transformer）。</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
           <t>摄影测量算法工程师</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
           <t>["多视几何","摄影测量","三维重建","SFM","密集匹配","光束平差","特征提取与匹配","畸变校正","多传感器融合","相机标定","LiDAR","C++","Python","OpenCV","OpenMVS","GPU加速","PyTorch","CNN","Transformer"]</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
           <t>["多视几何与摄影测量算法实现","多传感器融合与联合标定","AI 与传统方法结合优化处理流程"]</t>
@@ -3062,7 +2847,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V26" t="inlineStr"/>
       <c r="W26" t="inlineStr">
         <is>
           <t>title 按标题为摄影测量算法工程师（终审口径：级别不保留，去『高级』）；SIFT/SURF/ORB 并入特征提取与匹配；无年限；本科（硕士优先）</t>
@@ -3128,37 +2912,31 @@
 6. 熟悉编码规范能够写出简洁、易维护、可扩展的代码。</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
           <t>React前端工程师</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>["React","HTML5","CSS3","JavaScript","Webpack","Babel","前端性能优化"]</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
           <t>{"min_years":3,"max_years":null}</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
           <t>["React 前端开发与跨平台适配","性能与体验优化","前后端接口对接与代码维护"]</t>
@@ -3169,7 +2947,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr">
         <is>
           <t>title 保留 React 细化（终审口径：移除泛化『前端工程师』，保留『React前端工程师』格式）；3 年+；本科</t>
@@ -3240,29 +3017,21 @@
 4.有上线产品或项目作品可展示者优先。</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
           <t>前端工程师</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>["Android开发","Vue","uni-app","HTML5","CSS3","JavaScript"]</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr">
         <is>
           <t>["iOS开发","微信小程序开发","混合开发","UI设计"]</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
           <t>["移动端与 Web 前端开发维护","前端架构设计与组件化开发","页面实现与接口联调"]</t>
@@ -3273,7 +3042,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr">
         <is>
           <t>title 按终审口径细化：移除泛化『前端工程师』，主框架 Vue/uniapp → Vue前端工程师；skills 6 项；无学历/年限条款 | 口径修订 08-14：标题无细分词不保留正文细分（标题含细分词才保留，对齐 r2_014）</t>
@@ -3349,37 +3117,31 @@
 </t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
           <t>全栈开发工程师</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>["JavaScript","Java","Vue","Spring Boot","Spring Cloud","MySQL","PostgreSQL","Redis","MongoDB","RabbitMQ","Kafka","RocketMQ","Maven","Gradle","Git","Linux","SQL"]</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr">
         <is>
           <t>["Dubbo","gRPC","微服务","Docker","Kubernetes","分布式事务","分库分表","阿里云","腾讯云","AWS"]</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
           <t>{"min_years":1,"max_years":null}</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
           <t>["核心产品需求分析与系统设计","全栈编码实现与模块测试","系统架构讨论与性能优化"]</t>
@@ -3390,7 +3152,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr">
         <is>
           <t>title 与草稿一致；skills 17 项；1 年+；本科</t>
@@ -3458,29 +3219,21 @@
 </t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
           <t>AI全栈工程师</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>["LLM","VLM","客户端开发","RAG","Agent","知识库构建","Python","Java","Go","CI/CD","UI设计","Figma"]</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
           <t>["AI 智能体客户端开发与端侧 LLM/VLM 落地","客户端 CI/CD 与稳定性治理","UI/UX 设计实现","RAG/Agent 后端工程化"]</t>
@@ -3491,7 +3244,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr">
         <is>
           <t>⚠️ title 修正：草稿『客户端开发工程师』按标题为 AI全栈工程师（职责为客户端+UI+后端三方向）；正文无任职要求节，skills 按职责推导，学历/年限留空</t>
@@ -3569,37 +3321,31 @@
 </t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
           <t>Python工程师</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>["Python","高性能计算","并行计算","多线程","并发编程","异步编程","MySQL","PostgreSQL","Git"]</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr">
         <is>
           <t>["AWS","GCP","Azure","Django","Flask","FastAPI","单元测试"]</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
           <t>{"min_years":2,"max_years":null}</t>
         </is>
       </c>
-      <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
           <t>["计算金融应用开发","高性能并行计算优化","金融模型与仿真集成","API 与库实现"]</t>
@@ -3610,7 +3356,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V31" t="inlineStr"/>
       <c r="W31" t="inlineStr">
         <is>
           <t>⚠️ title：草稿『计算金融软件工程师』为正文语义，按招聘标题为 Python工程师（英文 JD）；2 年+；本科/硕士</t>
@@ -3679,37 +3424,31 @@
 9.工作积极主动，责任心强，拥有良好团队协作意识与沟通能力。</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr">
         <is>
           <t>Java后端工程师</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>["Java","Spring Boot","Dubbo","Thrift","Redis","RabbitMQ","Kafka","RocketMQ","达梦数据库","SQL","存储过程","ORM","RESTful API"]</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
           <t>{"min_years":1,"max_years":2}</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
           <t>本科</t>
         </is>
       </c>
-      <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
           <t>["信息化产品后端开发与接口设计","数据库设计与 SQL 优化","接口联调与系统优化"]</t>
@@ -3720,7 +3459,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V32" t="inlineStr"/>
       <c r="W32" t="inlineStr">
         <is>
           <t>⚠️ title：草稿加『开发』二字，按标题为 Java后端工程师（大小写规范）；1-2 年；本科；前端基础『优先』过泛不入 bonus</t>
@@ -3813,37 +3551,31 @@
 - 具有机器人相关项目经验者优先</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
           <t>机器视觉算法工程师</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>["目标检测","目标跟踪","图像分割","人脸识别","表情分析","人体姿态估计","OCR","视频动作检测","视频行为理解","多模态大模型","少样本学习","度量学习","迁移学习","自监督学习","OpenCV","C/C++","Python","Linux","ONNX","RKNN","模型量化","嵌入式部署"]</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr">
         <is>
           <t>["TensorRT","NCNN","MNN","OpenVINO","LLM","VLM","强化学习","ISP"]</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
           <t>{"min_years":3,"max_years":null}</t>
         </is>
       </c>
-      <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
           <t>硕士</t>
         </is>
       </c>
-      <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
           <t>["仿生机器人视觉算法研发","多模态大模型算法设计与落地","嵌入式部署与性能优化","图像处理链路设计"]</t>
@@ -3854,7 +3586,6 @@
           <t>人工终审_定稿</t>
         </is>
       </c>
-      <c r="V33" t="inlineStr"/>
       <c r="W33" t="inlineStr">
         <is>
           <t>⚠️ title：草稿『机器视觉算法工程师』，正文自述亦为机器视觉——按招聘标题为视觉算法工程师（终审可改）；22 项 skills；3 年+；硕士</t>

</xml_diff>